<commit_message>
Lock database function grants to an explicit allowlist (B1)
notify_household, send_push_for_notification and ensure_period were
callable by anyone with the publishable key, because functions created
after 0004's one-time revoke kept the default EXECUTE-to-PUBLIC grant.
0034 revokes EXECUTE on every non-extension function in public, grants
back only what the app, RLS policies and views need, closes default
privileges for future functions, and makes ensure_period refuse other
households. Security tests now require a 42501 refusal for internals.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/roomly-production-readiness.xlsx
+++ b/docs/roomly-production-readiness.xlsx
@@ -949,12 +949,16 @@
       </c>
       <c r="J2" s="15" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K2" s="15" t="inlineStr"/>
       <c r="L2" s="16" t="inlineStr"/>
-      <c r="M2" s="15" t="inlineStr"/>
+      <c r="M2" s="15" t="inlineStr">
+        <is>
+          <t>Migration 0034 applied 2026-10-10; security tests 38/38.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">

</xml_diff>